<commit_message>
data: atualização CME Futures 2026-06-22
</commit_message>
<xml_diff>
--- a/data/CME_Futures_Database.xlsx
+++ b/data/CME_Futures_Database.xlsx
@@ -507,7 +507,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>3.198</t>
+          <t>3.305</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -534,7 +534,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>3.247</t>
+          <t>3.341</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -561,7 +561,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>3.207</t>
+          <t>3.296</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -588,7 +588,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>3.240</t>
+          <t>3.326</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -615,7 +615,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>3.435</t>
+          <t>3.511</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -642,7 +642,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>4.049</t>
+          <t>4.115</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -669,7 +669,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>4.454</t>
+          <t>4.513</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -696,7 +696,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>4.026</t>
+          <t>4.077</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -723,7 +723,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>3.202</t>
+          <t>3.246</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -750,7 +750,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2.975</t>
+          <t>3.015</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -777,7 +777,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2.957</t>
+          <t>2.987</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>3.098</t>
+          <t>3.123</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -831,7 +831,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>3.311</t>
+          <t>3.333</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -858,7 +858,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>3.367</t>
+          <t>3.387</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -885,7 +885,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>3.344</t>
+          <t>3.362</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -912,7 +912,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>3.417</t>
+          <t>3.437</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -939,7 +939,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>3.674</t>
+          <t>3.686</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>4.317</t>
+          <t>4.324</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -993,7 +993,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>4.733</t>
+          <t>4.735</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1020,7 +1020,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>4.250</t>
+          <t>4.257</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1047,7 +1047,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1074,7 +1074,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1101,7 +1101,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>3.141</t>
+          <t>3.151</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1128,7 +1128,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>3.279</t>
+          <t>3.290</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>3.488</t>
+          <t>3.511</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1182,7 +1182,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>3.548</t>
+          <t>3.563</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1209,7 +1209,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>3.528</t>
+          <t>3.533</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1236,7 +1236,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>3.594</t>
+          <t>3.617</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1263,7 +1263,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>3.806</t>
+          <t>3.825</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1290,7 +1290,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>4.394</t>
+          <t>4.410</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1317,7 +1317,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1344,7 +1344,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1398,7 +1398,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1425,7 +1425,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1452,7 +1452,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1479,7 +1479,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1506,7 +1506,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1533,7 +1533,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1560,7 +1560,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1587,7 +1587,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1614,7 +1614,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1641,7 +1641,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1668,7 +1668,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1722,7 +1722,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1749,7 +1749,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1776,7 +1776,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1803,7 +1803,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -1830,7 +1830,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1857,7 +1857,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1884,7 +1884,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -1911,7 +1911,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -1938,7 +1938,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -1965,7 +1965,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -1992,7 +1992,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -2019,7 +2019,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2046,7 +2046,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -2073,7 +2073,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2100,7 +2100,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -2127,7 +2127,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -2181,7 +2181,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2208,7 +2208,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -2235,7 +2235,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2262,7 +2262,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -2289,7 +2289,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2316,7 +2316,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -2343,7 +2343,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2370,7 +2370,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -2397,7 +2397,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -2451,7 +2451,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2478,7 +2478,7 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -2505,7 +2505,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2532,7 +2532,7 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -2559,7 +2559,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -2613,7 +2613,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2640,7 +2640,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -2667,7 +2667,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2694,7 +2694,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -2721,7 +2721,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2748,7 +2748,7 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -2775,7 +2775,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -2802,7 +2802,7 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -2829,7 +2829,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -2856,7 +2856,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -2883,7 +2883,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -2910,7 +2910,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -2937,7 +2937,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -2964,7 +2964,7 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -2991,7 +2991,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -3018,7 +3018,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -3045,7 +3045,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -3072,7 +3072,7 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -3099,7 +3099,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -3126,7 +3126,7 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -3153,7 +3153,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3180,7 +3180,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -3256,7 +3256,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -3283,7 +3283,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3310,7 +3310,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -3337,7 +3337,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -3364,7 +3364,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -3391,7 +3391,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -3418,7 +3418,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -3445,7 +3445,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -3472,7 +3472,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -3499,7 +3499,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -3526,7 +3526,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -3553,7 +3553,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -3580,7 +3580,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -3607,7 +3607,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -3634,7 +3634,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -3661,7 +3661,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -3688,7 +3688,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -3715,7 +3715,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -3742,7 +3742,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -3769,7 +3769,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -3796,7 +3796,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -3823,7 +3823,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -3850,7 +3850,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -3877,7 +3877,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -3904,7 +3904,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -3931,7 +3931,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -3958,7 +3958,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3985,7 +3985,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -4012,7 +4012,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -4039,7 +4039,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -4066,7 +4066,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -4093,7 +4093,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -4120,7 +4120,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -4147,7 +4147,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -4174,7 +4174,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -4201,7 +4201,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -4228,7 +4228,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -4255,7 +4255,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -4282,7 +4282,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -4309,7 +4309,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -4336,7 +4336,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -4363,7 +4363,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -4390,7 +4390,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -4417,7 +4417,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -4444,7 +4444,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4471,7 +4471,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -4498,7 +4498,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -4525,7 +4525,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -4552,7 +4552,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -4579,7 +4579,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -4606,7 +4606,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -4633,7 +4633,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -4660,7 +4660,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -4687,7 +4687,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -4714,7 +4714,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -4741,7 +4741,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -4768,7 +4768,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -4795,7 +4795,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -4822,7 +4822,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -4849,7 +4849,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -4876,7 +4876,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -4903,7 +4903,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -4930,7 +4930,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -4957,7 +4957,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -4984,7 +4984,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -5011,7 +5011,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -5038,7 +5038,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -5065,7 +5065,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -5092,7 +5092,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -5119,7 +5119,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -5146,7 +5146,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -5173,7 +5173,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -5200,7 +5200,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -5227,7 +5227,7 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -5254,7 +5254,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -5281,7 +5281,7 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -5308,7 +5308,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -5335,7 +5335,7 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -5362,7 +5362,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -5389,7 +5389,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -5416,7 +5416,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -5443,7 +5443,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -5470,7 +5470,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -5497,7 +5497,7 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -5524,7 +5524,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -5551,7 +5551,7 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -5578,7 +5578,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -5605,7 +5605,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -5632,7 +5632,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -5708,7 +5708,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -5735,7 +5735,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -5762,7 +5762,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -5789,7 +5789,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -5816,7 +5816,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -5843,7 +5843,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -5870,7 +5870,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -5924,7 +5924,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -5951,7 +5951,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -5978,7 +5978,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -6005,7 +6005,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -6032,7 +6032,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -6059,7 +6059,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -6086,7 +6086,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -6113,7 +6113,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -6140,7 +6140,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -6194,7 +6194,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -6221,7 +6221,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -6248,7 +6248,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -6275,7 +6275,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -6302,7 +6302,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -6329,7 +6329,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -6356,7 +6356,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -6383,7 +6383,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -6410,7 +6410,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -6464,7 +6464,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -6491,7 +6491,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -6518,7 +6518,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -6545,7 +6545,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -6572,7 +6572,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -6599,7 +6599,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -6626,7 +6626,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -6653,7 +6653,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -6680,7 +6680,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -6734,7 +6734,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -6761,7 +6761,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -6788,7 +6788,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -6815,7 +6815,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -6842,7 +6842,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -6869,7 +6869,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -6896,7 +6896,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -6923,7 +6923,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -6950,7 +6950,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -7004,7 +7004,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -7031,7 +7031,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -7058,7 +7058,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -7085,7 +7085,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -7112,7 +7112,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -7139,7 +7139,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -7166,7 +7166,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -7193,7 +7193,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -7220,7 +7220,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -7274,7 +7274,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -7301,7 +7301,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -7328,7 +7328,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -7355,7 +7355,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -7382,7 +7382,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -7409,7 +7409,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -7436,7 +7436,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -7463,7 +7463,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -7539,7 +7539,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -7566,7 +7566,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -7593,7 +7593,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -7620,7 +7620,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -7647,7 +7647,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -7674,7 +7674,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -7701,7 +7701,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -7728,7 +7728,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -7755,7 +7755,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -7782,7 +7782,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -7809,7 +7809,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -7836,7 +7836,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -7863,7 +7863,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -7890,7 +7890,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -7917,7 +7917,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -7944,7 +7944,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -7971,7 +7971,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -7998,7 +7998,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -8025,7 +8025,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -8052,7 +8052,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -8079,7 +8079,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -8106,7 +8106,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -8133,7 +8133,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -8160,7 +8160,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -8187,7 +8187,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -8214,7 +8214,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -8241,7 +8241,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -8268,7 +8268,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -8295,7 +8295,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -8322,7 +8322,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -8349,7 +8349,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -8376,7 +8376,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -8403,7 +8403,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -8430,7 +8430,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -8457,7 +8457,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -8484,7 +8484,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -8511,7 +8511,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -8538,7 +8538,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -8565,7 +8565,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -8592,7 +8592,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -8619,7 +8619,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -8646,7 +8646,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -8673,7 +8673,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -8700,7 +8700,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -8727,7 +8727,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -8754,7 +8754,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -8781,7 +8781,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -8808,7 +8808,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -8835,7 +8835,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -8862,7 +8862,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -8889,7 +8889,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -8916,7 +8916,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -8943,7 +8943,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -8970,7 +8970,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -8997,7 +8997,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -9024,7 +9024,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -9051,7 +9051,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -9078,7 +9078,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -9105,7 +9105,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -9132,7 +9132,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -9159,7 +9159,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -9186,7 +9186,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -9213,7 +9213,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -9240,7 +9240,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -9267,7 +9267,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -9294,7 +9294,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -9370,7 +9370,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -9385,7 +9385,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>42.070</t>
+          <t>42.610</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -9397,7 +9397,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -9412,7 +9412,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>40.648</t>
+          <t>41.775</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -9424,7 +9424,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -9451,7 +9451,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -9478,7 +9478,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -9505,7 +9505,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -9532,7 +9532,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -9559,7 +9559,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -9586,7 +9586,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -9613,7 +9613,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -9640,7 +9640,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -9667,7 +9667,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -9694,7 +9694,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -9721,7 +9721,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -9748,7 +9748,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -9775,7 +9775,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -9802,7 +9802,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -9829,7 +9829,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -9856,7 +9856,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -9883,7 +9883,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -9910,7 +9910,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -9937,7 +9937,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -9964,7 +9964,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -9991,7 +9991,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -10018,7 +10018,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -10045,7 +10045,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -10072,7 +10072,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -10099,7 +10099,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -10126,7 +10126,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -10153,7 +10153,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -10180,7 +10180,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -10207,7 +10207,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -10234,7 +10234,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -10261,7 +10261,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -10288,7 +10288,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -10315,7 +10315,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -10342,7 +10342,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -10369,7 +10369,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -10396,7 +10396,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -10423,7 +10423,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -10450,7 +10450,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -10477,7 +10477,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -10504,7 +10504,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -10531,7 +10531,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -10558,7 +10558,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -10585,7 +10585,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -10612,7 +10612,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -10639,7 +10639,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -10666,7 +10666,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -10693,7 +10693,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -10720,7 +10720,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -10747,7 +10747,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -10774,7 +10774,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -10801,7 +10801,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -10828,7 +10828,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -10855,7 +10855,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -10882,7 +10882,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -10909,7 +10909,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -10936,7 +10936,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -10963,7 +10963,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -10990,7 +10990,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -11017,7 +11017,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -11044,7 +11044,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -11071,7 +11071,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -11098,7 +11098,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -11125,7 +11125,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -11152,7 +11152,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -11179,7 +11179,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -11206,7 +11206,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -11233,7 +11233,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -11260,7 +11260,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -11287,7 +11287,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -11314,7 +11314,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -11341,7 +11341,7 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -11368,7 +11368,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -11395,7 +11395,7 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -11422,7 +11422,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -11449,7 +11449,7 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -11476,7 +11476,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -11503,7 +11503,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -11530,7 +11530,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -11557,7 +11557,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -11584,7 +11584,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -11611,7 +11611,7 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -11638,7 +11638,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -11665,7 +11665,7 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -11692,7 +11692,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -11719,7 +11719,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -11746,7 +11746,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -11773,7 +11773,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -11800,7 +11800,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -11827,7 +11827,7 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -11854,7 +11854,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -11881,7 +11881,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -11908,7 +11908,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -11935,7 +11935,7 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -11962,7 +11962,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -11989,7 +11989,7 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -12016,7 +12016,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -12043,7 +12043,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: backfill cotações diárias junho
</commit_message>
<xml_diff>
--- a/data/CME_Futures_Database.xlsx
+++ b/data/CME_Futures_Database.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HH" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Brent" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="NBP" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="JKM" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TTF" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cotações Diárias" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="HH" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Brent" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="NBP" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="JKM" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="TTF" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +39,10 @@
     <font>
       <name val="Arial"/>
       <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -90,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -99,6 +104,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -463,6 +477,818 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E86AB"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>HH</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Brent</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>NBP</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>JKM</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>TTF</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Coal_API2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>3.1790</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>94.9800</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>119.0900</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>18.6850</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>49.0900</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>3.1670</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>96.0000</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>114.7900</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>18.6100</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>47.6070</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>3.2140</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>97.8100</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>117.9000</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>18.8150</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>48.8640</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>3.3360</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>95.0300</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>117.9300</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>18.7650</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>48.7520</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>3.2290</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>93.0900</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>117.0500</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>18.7750</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>48.4960</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>3.1470</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>94.2500</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>120.5300</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>18.8950</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>49.8260</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>3.1400</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>91.4500</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>117.1900</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>18.8850</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>48.7440</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>3.1850</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>93.1000</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>120.3200</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>18.9150</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>49.9890</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>3.0870</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>90.3800</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>119.7600</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>18.9200</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>49.6900</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>3.1200</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>87.3300</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>111.9100</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>18.8550</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>46.7730</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>3.1470</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>83.1700</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>101.0100</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>18.7830</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>42.5070</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>3.2390</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>78.9600</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>99.4000</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>15.9400</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>41.7690</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>3.1450</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>79.5500</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>99.7800</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>15.8200</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>41.9150</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>3.2330</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>79.8500</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>96.6900</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>15.3150</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>40.5230</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>3.2530</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>77.9000</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>99.9400</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>15.8600</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>41.8870</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>3.1470</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>77.0800</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>100.2900</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>15.7400</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>42.0140</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>3.2210</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>73.7400</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>97.1800</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>15.5500</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>40.8760</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>3.3430</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>75.2600</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>96.5200</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>15.3850</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>40.4050</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>3.2310</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>71.9900</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>97.8000</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>15.5250</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>40.7820</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>3.1810</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>73.1500</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>102.6100</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>15.8200</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>42.5650</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>3.2750</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>72.9200</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>104.4500</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>16.0500</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>43.4440</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>3.2200</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>71.5700</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>101.6900</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>16.0250</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>42.7790</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>3.1640</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>70.8000</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>43.9950</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="001F4E79"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -8609,7 +9435,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00833C00"/>
@@ -15867,7 +16693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00375623"/>
@@ -21262,7 +22088,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -26603,7 +27429,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C55A11"/>

</xml_diff>

<commit_message>
fix: cotações diárias sem Coal_API2, datas recentes primeiro
</commit_message>
<xml_diff>
--- a/data/CME_Futures_Database.xlsx
+++ b/data/CME_Futures_Database.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -490,7 +490,6 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -524,374 +523,350 @@
           <t>TTF</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Coal_API2</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>3.1790</t>
+          <t>3.1910</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>94.9800</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>119.0900</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>18.6850</t>
-        </is>
-      </c>
+          <t>70.7000</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr"/>
+      <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>49.0900</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr"/>
+          <t>43.9950</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>3.1670</t>
+          <t>3.2200</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>96.0000</t>
+          <t>71.5700</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>114.7900</t>
+          <t>101.6900</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>18.6100</t>
+          <t>16.0250</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>47.6070</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr"/>
+          <t>42.7790</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>3.2140</t>
+          <t>3.2750</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>97.8100</t>
+          <t>72.9200</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>117.9000</t>
+          <t>104.4500</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>18.8150</t>
+          <t>16.0500</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>48.8640</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr"/>
+          <t>43.4440</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>3.3360</t>
+          <t>3.1810</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>95.0300</t>
+          <t>73.1500</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>117.9300</t>
+          <t>102.6100</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>18.7650</t>
+          <t>15.8200</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>48.7520</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr"/>
+          <t>42.5650</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>3.2290</t>
+          <t>3.2310</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>93.0900</t>
+          <t>71.9900</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>117.0500</t>
+          <t>97.8000</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>18.7750</t>
+          <t>15.5250</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>48.4960</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
+          <t>40.7820</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>3.1470</t>
+          <t>3.3430</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>94.2500</t>
+          <t>75.2600</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>120.5300</t>
+          <t>96.5200</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>18.8950</t>
+          <t>15.3850</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>49.8260</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr"/>
+          <t>40.4050</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>3.1400</t>
+          <t>3.2210</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>91.4500</t>
+          <t>73.7400</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>117.1900</t>
+          <t>97.1800</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>18.8850</t>
+          <t>15.5500</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>48.7440</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr"/>
+          <t>40.8760</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>3.1850</t>
+          <t>3.1470</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>93.1000</t>
+          <t>77.0800</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>120.3200</t>
+          <t>100.2900</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>18.9150</t>
+          <t>15.7400</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>49.9890</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr"/>
+          <t>42.0140</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>3.0870</t>
+          <t>3.2530</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>90.3800</t>
+          <t>77.9000</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>119.7600</t>
+          <t>99.9400</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>18.9200</t>
+          <t>15.8600</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>49.6900</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr"/>
+          <t>41.8870</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>3.1200</t>
+          <t>3.2330</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>87.3300</t>
+          <t>79.8500</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>111.9100</t>
+          <t>96.6900</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>18.8550</t>
+          <t>15.3150</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>46.7730</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr"/>
+          <t>40.5230</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>3.1470</t>
+          <t>3.1450</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>83.1700</t>
+          <t>79.5500</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>101.0100</t>
+          <t>99.7800</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>18.7830</t>
+          <t>15.8200</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>42.5070</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr"/>
+          <t>41.9150</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -924,362 +899,358 @@
           <t>41.7690</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>3.1450</t>
+          <t>3.1470</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>79.5500</t>
+          <t>83.1700</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>99.7800</t>
+          <t>101.0100</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>15.8200</t>
+          <t>18.7830</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>41.9150</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr"/>
+          <t>42.5070</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>3.2330</t>
+          <t>3.1200</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>79.8500</t>
+          <t>87.3300</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>96.6900</t>
+          <t>111.9100</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>15.3150</t>
+          <t>18.8550</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>40.5230</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr"/>
+          <t>46.7730</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>3.2530</t>
+          <t>3.0870</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>77.9000</t>
+          <t>90.3800</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>99.9400</t>
+          <t>119.7600</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>15.8600</t>
+          <t>18.9200</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>41.8870</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr"/>
+          <t>49.6900</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>3.1470</t>
+          <t>3.1850</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>77.0800</t>
+          <t>93.1000</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>100.2900</t>
+          <t>120.3200</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>15.7400</t>
+          <t>18.9150</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>42.0140</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr"/>
+          <t>49.9890</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>3.2210</t>
+          <t>3.1400</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>73.7400</t>
+          <t>91.4500</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>97.1800</t>
+          <t>117.1900</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>15.5500</t>
+          <t>18.8850</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>40.8760</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr"/>
+          <t>48.7440</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>3.3430</t>
+          <t>3.1470</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>75.2600</t>
+          <t>94.2500</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>96.5200</t>
+          <t>120.5300</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>15.3850</t>
+          <t>18.8950</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>40.4050</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr"/>
+          <t>49.8260</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>3.2310</t>
+          <t>3.2290</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>71.9900</t>
+          <t>93.0900</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>97.8000</t>
+          <t>117.0500</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>15.5250</t>
+          <t>18.7750</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>40.7820</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr"/>
+          <t>48.4960</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>3.1810</t>
+          <t>3.3360</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>73.1500</t>
+          <t>95.0300</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>102.6100</t>
+          <t>117.9300</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>15.8200</t>
+          <t>18.7650</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>42.5650</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr"/>
+          <t>48.7520</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>3.2750</t>
+          <t>3.2140</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>72.9200</t>
+          <t>97.8100</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>104.4500</t>
+          <t>117.9000</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>16.0500</t>
+          <t>18.8150</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>43.4440</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr"/>
+          <t>48.8640</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>3.2200</t>
+          <t>3.1670</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>71.5700</t>
+          <t>96.0000</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>101.6900</t>
+          <t>114.7900</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>16.0250</t>
+          <t>18.6100</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>42.7790</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr"/>
+          <t>47.6070</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>3.1910</t>
+          <t>3.1790</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>70.7000</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr"/>
-      <c r="E24" s="5" t="inlineStr"/>
+          <t>94.9800</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>119.0900</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>18.6850</t>
+        </is>
+      </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>43.9950</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr"/>
+          <t>49.0900</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>